<commit_message>
More clean up and segregation of agents.
</commit_message>
<xml_diff>
--- a/OLD--_OUTPUT--Recruiting_Coord.xlsx
+++ b/OLD--_OUTPUT--Recruiting_Coord.xlsx
@@ -643,7 +643,7 @@
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Dim6_RecruitingOps_Score (0-3)</t>
+          <t>Dim6_RecruitingOps_Score (0-4)</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
@@ -17074,7 +17074,7 @@
       </c>
       <c r="J107" s="10" t="inlineStr">
         <is>
-          <t>LinkedIn Recruiter access denied - profile ID AEMAAC56J-wBJLXiiRndjJJwPZq4Ekc0CwoPY4MM not accessible</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K107" s="10" t="n">
@@ -17150,10 +17150,14 @@
       </c>
       <c r="AJ107" s="10" t="inlineStr">
         <is>
-          <t>Unable to Evaluate</t>
-        </is>
-      </c>
-      <c r="AK107" s="10" t="n"/>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="AK107" s="10" t="inlineStr">
+        <is>
+          <t>Hard No</t>
+        </is>
+      </c>
       <c r="AL107" s="10" t="n"/>
       <c r="AM107" s="10" t="n"/>
       <c r="AN107" s="10" t="inlineStr">
@@ -43066,7 +43070,7 @@
       </c>
       <c r="AK268" s="15" t="inlineStr">
         <is>
-          <t>Hard No — Auto-DQ</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL268" s="15" t="inlineStr"/>
@@ -43192,7 +43196,7 @@
       </c>
       <c r="AK269" s="15" t="inlineStr">
         <is>
-          <t>Hard No — Auto-DQ</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL269" s="15" t="inlineStr"/>
@@ -43318,7 +43322,7 @@
       </c>
       <c r="AK270" s="15" t="inlineStr">
         <is>
-          <t>Hard No — Auto-DQ</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL270" s="15" t="inlineStr"/>
@@ -43444,7 +43448,7 @@
       </c>
       <c r="AK271" s="15" t="inlineStr">
         <is>
-          <t>Hard No — Auto-DQ</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL271" s="15" t="inlineStr"/>
@@ -43736,7 +43740,7 @@
       </c>
       <c r="AK273" s="15" t="inlineStr">
         <is>
-          <t>Hard No — Auto-DQ</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL273" s="15" t="inlineStr"/>
@@ -43862,7 +43866,7 @@
       </c>
       <c r="AK274" s="15" t="inlineStr">
         <is>
-          <t>Hard No — non-tech traditional industry recruiting (pharma mfg, coal &amp; mining, finance)</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL274" s="15" t="inlineStr"/>
@@ -44020,7 +44024,7 @@
       </c>
       <c r="AK275" s="15" t="inlineStr">
         <is>
-          <t>Strong Yes — exact RC title at Lendingkart fintech (2yr), 3500-candidate high-volume hiring, Darwinbox + Greenhouse ATS, sales hiring experience</t>
+          <t>Strong Yes</t>
         </is>
       </c>
       <c r="AL275" s="15" t="inlineStr">
@@ -44154,7 +44158,7 @@
       </c>
       <c r="AK276" s="15" t="inlineStr">
         <is>
-          <t>Hard No — pure agency staffing (REQ Solutions) with healthcare sourcing, no in-house experience</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL276" s="15" t="inlineStr"/>
@@ -44280,7 +44284,7 @@
       </c>
       <c r="AK277" s="15" t="inlineStr">
         <is>
-          <t>Hard No — pure agency staffing chain (Veterans Sourcing Group + IMS People Possible)</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL277" s="15" t="inlineStr"/>
@@ -44406,7 +44410,7 @@
       </c>
       <c r="AK278" s="15" t="inlineStr">
         <is>
-          <t>Hard No — pure agency staffing (Placon HR Services), no in-house experience, still pursuing MBA</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL278" s="15" t="inlineStr"/>
@@ -44532,7 +44536,7 @@
       </c>
       <c r="AK279" s="15" t="inlineStr">
         <is>
-          <t>Hard No — pure RPO agency (Horizon Talent Alliance), serving US staffing firms offshore</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL279" s="15" t="inlineStr"/>
@@ -44658,7 +44662,7 @@
       </c>
       <c r="AK280" s="15" t="inlineStr">
         <is>
-          <t>Hard No — pure agency (iConsultera), healthcare staffing, accounting industry</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL280" s="15" t="inlineStr"/>
@@ -44784,7 +44788,7 @@
       </c>
       <c r="AK281" s="15" t="inlineStr">
         <is>
-          <t>Hard No — pure agency chain (Confidential + LanceSoft), UK/Europe focus, contract/interim staffing</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL281" s="15" t="inlineStr"/>
@@ -44942,7 +44946,7 @@
       </c>
       <c r="AK282" s="15" t="inlineStr">
         <is>
-          <t>Hard No — very junior TA at legal services company, no high-volume/SaaS/sales hiring experience</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL282" s="15" t="inlineStr">
@@ -45076,7 +45080,7 @@
       </c>
       <c r="AK283" s="15" t="inlineStr">
         <is>
-          <t>Hard No — pure agency chain (TalentCore + IMS Group), US IT staffing/bench sales</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL283" s="15" t="inlineStr"/>
@@ -45202,7 +45206,7 @@
       </c>
       <c r="AK284" s="15" t="inlineStr">
         <is>
-          <t>Hard No — BPO background (Medusind AR Caller) + IMS People Possible agency chain</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL284" s="15" t="inlineStr"/>
@@ -45328,7 +45332,7 @@
       </c>
       <c r="AK285" s="15" t="inlineStr">
         <is>
-          <t>Hard No — pure agency (Kyara Consulting), single role, no in-house experience</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL285" s="15" t="inlineStr"/>
@@ -45454,7 +45458,7 @@
       </c>
       <c r="AK286" s="15" t="inlineStr">
         <is>
-          <t>Hard No — pure IMS People Possible agency (4yr+), UK staffing, no in-house experience</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL286" s="15" t="inlineStr"/>
@@ -45580,7 +45584,7 @@
       </c>
       <c r="AK287" s="15" t="inlineStr">
         <is>
-          <t>Hard No — pure IMS Group agency (2yr 5mo), UK staffing operations</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL287" s="15" t="inlineStr"/>
@@ -45739,12 +45743,12 @@
       </c>
       <c r="AJ288" s="15" t="inlineStr">
         <is>
-          <t>DQ/F</t>
+          <t>F</t>
         </is>
       </c>
       <c r="AK288" s="15" t="inlineStr">
         <is>
-          <t>Hard No — primarily a teacher (6yr+), brief agency recruiter stint, education industry</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL288" s="15" t="inlineStr"/>
@@ -45903,12 +45907,12 @@
       </c>
       <c r="AJ289" s="15" t="inlineStr">
         <is>
-          <t>DQ/F</t>
+          <t>F</t>
         </is>
       </c>
       <c r="AK289" s="15" t="inlineStr">
         <is>
-          <t>Hard No — pure agency chain (IMS People Possible + Unity Systems), UK healthcare staffing</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL289" s="15" t="inlineStr"/>
@@ -46067,12 +46071,12 @@
       </c>
       <c r="AJ290" s="15" t="inlineStr">
         <is>
-          <t>DQ/F</t>
+          <t>F</t>
         </is>
       </c>
       <c r="AK290" s="15" t="inlineStr">
         <is>
-          <t>Hard No — pure IMS Group agency (4yr 6mo), pharma domain staffing</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL290" s="15" t="inlineStr"/>
@@ -46231,12 +46235,12 @@
       </c>
       <c r="AJ291" s="15" t="inlineStr">
         <is>
-          <t>DQ/F</t>
+          <t>F</t>
         </is>
       </c>
       <c r="AK291" s="15" t="inlineStr">
         <is>
-          <t>Hard No — pure IMS People Possible (2yr 9mo), healthcare/manufacturing/automotive staffing</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL291" s="15" t="inlineStr"/>
@@ -46394,7 +46398,7 @@
       </c>
       <c r="AK292" s="15" t="inlineStr">
         <is>
-          <t>No — exact TA Coordinator title but only 4mo tenure, 17yr career gap, no relevant modern experience</t>
+          <t>No</t>
         </is>
       </c>
       <c r="AL292" s="15" t="inlineStr">
@@ -46561,12 +46565,12 @@
       </c>
       <c r="AJ293" s="15" t="inlineStr">
         <is>
-          <t>DQ/F</t>
+          <t>F</t>
         </is>
       </c>
       <c r="AK293" s="15" t="inlineStr">
         <is>
-          <t>Hard No — pure agency (Dangi Recruitment) + auto dealership sales background, very junior</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL293" s="15" t="inlineStr"/>
@@ -46891,12 +46895,12 @@
       </c>
       <c r="AJ295" s="15" t="inlineStr">
         <is>
-          <t>DQ/F</t>
+          <t>F</t>
         </is>
       </c>
       <c r="AK295" s="15" t="inlineStr">
         <is>
-          <t>Hard No — pure agency bench sales (Radiance Technologies), no recruiting background</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL295" s="15" t="inlineStr"/>
@@ -47053,12 +47057,12 @@
       </c>
       <c r="AJ296" s="15" t="inlineStr">
         <is>
-          <t>DQ/F</t>
+          <t>F</t>
         </is>
       </c>
       <c r="AK296" s="15" t="inlineStr">
         <is>
-          <t>Hard No — Auto-DQ</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL296" s="15" t="n"/>
@@ -47215,12 +47219,12 @@
       </c>
       <c r="AJ297" s="15" t="inlineStr">
         <is>
-          <t>DQ/F</t>
+          <t>F</t>
         </is>
       </c>
       <c r="AK297" s="15" t="inlineStr">
         <is>
-          <t>Hard No — Auto-DQ</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL297" s="15" t="n"/>
@@ -47377,12 +47381,12 @@
       </c>
       <c r="AJ298" s="15" t="inlineStr">
         <is>
-          <t>DQ/F</t>
+          <t>F</t>
         </is>
       </c>
       <c r="AK298" s="15" t="inlineStr">
         <is>
-          <t>Hard No — Auto-DQ</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL298" s="15" t="n"/>
@@ -47539,12 +47543,12 @@
       </c>
       <c r="AJ299" s="15" t="inlineStr">
         <is>
-          <t>DQ/F</t>
+          <t>F</t>
         </is>
       </c>
       <c r="AK299" s="15" t="inlineStr">
         <is>
-          <t>Hard No — Auto-DQ</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL299" s="15" t="n"/>
@@ -47722,8 +47726,10 @@
       </c>
     </row>
     <row r="301">
-      <c r="A301" t="n">
-        <v>300</v>
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Subhro Bose</t>
+        </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
@@ -47767,12 +47773,12 @@
       </c>
       <c r="J301" t="inlineStr">
         <is>
-          <t>Ahmedabad, Gujarat, India</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K301" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Row corrupted - data shifted, missing URLs</t>
         </is>
       </c>
       <c r="L301" t="inlineStr">
@@ -47800,109 +47806,64 @@
           <t>0</t>
         </is>
       </c>
-      <c r="Q301" t="inlineStr">
-        <is>
-          <t>Auto-DQ</t>
-        </is>
-      </c>
       <c r="R301" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="S301" t="inlineStr">
-        <is>
-          <t>Auto-DQ</t>
-        </is>
-      </c>
       <c r="T301" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="U301" t="inlineStr">
-        <is>
-          <t>Auto-DQ</t>
-        </is>
-      </c>
       <c r="V301" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="W301" t="inlineStr">
-        <is>
-          <t>Auto-DQ</t>
-        </is>
-      </c>
       <c r="X301" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="Y301" t="inlineStr">
-        <is>
-          <t>Auto-DQ</t>
-        </is>
-      </c>
       <c r="Z301" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AA301" t="inlineStr">
-        <is>
-          <t>Auto-DQ</t>
-        </is>
-      </c>
       <c r="AB301" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AC301" t="inlineStr">
-        <is>
-          <t>Auto-DQ</t>
-        </is>
-      </c>
-      <c r="AD301" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AE301" t="inlineStr">
-        <is>
-          <t>Auto-DQ</t>
-        </is>
-      </c>
-      <c r="AF301" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AG301" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AH301" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="AD301" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE301" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF301" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG301" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH301" t="n">
+        <v>53.4</v>
       </c>
       <c r="AI301" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ301" t="inlineStr">
         <is>
-          <t>53.4</t>
+          <t>F</t>
         </is>
       </c>
       <c r="AK301" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL301" t="inlineStr">
@@ -47913,6 +47874,11 @@
       <c r="AM301" t="inlineStr">
         <is>
           <t>Hard No</t>
+        </is>
+      </c>
+      <c r="AN301" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -47986,12 +47952,26 @@
       <c r="AA302" s="15" t="inlineStr"/>
       <c r="AB302" s="15" t="inlineStr"/>
       <c r="AC302" s="15" t="inlineStr"/>
-      <c r="AD302" s="15" t="inlineStr"/>
-      <c r="AE302" s="15" t="inlineStr"/>
-      <c r="AF302" s="15" t="inlineStr"/>
-      <c r="AG302" s="15" t="inlineStr"/>
-      <c r="AH302" s="15" t="inlineStr"/>
-      <c r="AI302" s="15" t="inlineStr"/>
+      <c r="AD302" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE302" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF302" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG302" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH302" s="15" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="AI302" s="15" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
       <c r="AJ302" s="15" t="inlineStr">
         <is>
           <t>F</t>
@@ -48004,7 +47984,11 @@
       </c>
       <c r="AL302" s="15" t="inlineStr"/>
       <c r="AM302" s="15" t="inlineStr"/>
-      <c r="AN302" s="15" t="inlineStr"/>
+      <c r="AN302" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="15" t="inlineStr">
@@ -48112,34 +48096,24 @@
         </is>
       </c>
       <c r="AC303" s="15" t="inlineStr"/>
-      <c r="AD303" s="15" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="AE303" s="15" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="AF303" s="15" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="AG303" s="15" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="AH303" s="15" t="inlineStr">
-        <is>
-          <t>53.4</t>
-        </is>
+      <c r="AD303" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE303" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF303" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG303" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH303" s="15" t="n">
+        <v>53.4</v>
       </c>
       <c r="AI303" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ303" s="15" t="inlineStr">
@@ -48154,7 +48128,11 @@
       </c>
       <c r="AL303" s="15" t="inlineStr"/>
       <c r="AM303" s="15" t="inlineStr"/>
-      <c r="AN303" s="15" t="inlineStr"/>
+      <c r="AN303" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="15" t="inlineStr">
@@ -48276,27 +48254,43 @@
           <t>ZURU appears growth-stage tech but no explicit VC/YC mention; Ascension is large enterprise; minimal startup experience</t>
         </is>
       </c>
-      <c r="AD304" s="15" t="inlineStr">
+      <c r="AD304" s="15" t="n">
+        <v>26.33333333333334</v>
+      </c>
+      <c r="AE304" s="15" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="AF304" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="AG304" s="15" t="n">
+        <v>29.93333333333334</v>
+      </c>
+      <c r="AH304" s="15" t="n">
+        <v>53.4</v>
+      </c>
+      <c r="AI304" s="15" t="inlineStr">
+        <is>
+          <t>56.1%</t>
+        </is>
+      </c>
+      <c r="AJ304" s="15" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="AE304" s="15" t="inlineStr">
+      <c r="AK304" s="15" t="inlineStr">
         <is>
           <t>Maybe</t>
         </is>
       </c>
-      <c r="AF304" s="15" t="n">
-        <v>56.93</v>
-      </c>
-      <c r="AG304" s="15" t="inlineStr"/>
-      <c r="AH304" s="15" t="inlineStr"/>
-      <c r="AI304" s="15" t="inlineStr"/>
-      <c r="AJ304" s="15" t="inlineStr"/>
-      <c r="AK304" s="15" t="inlineStr"/>
       <c r="AL304" s="15" t="inlineStr"/>
       <c r="AM304" s="15" t="inlineStr"/>
-      <c r="AN304" s="15" t="inlineStr"/>
+      <c r="AN304" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="15" t="inlineStr">
@@ -48452,10 +48446,8 @@
           <t>26.4</t>
         </is>
       </c>
-      <c r="AH305" s="15" t="inlineStr">
-        <is>
-          <t>53.4</t>
-        </is>
+      <c r="AH305" s="15" t="n">
+        <v>53.4</v>
       </c>
       <c r="AI305" s="15" t="inlineStr">
         <is>
@@ -48486,7 +48478,11 @@
           <t>No demonstrated Sales role hiring experience (critical for SwiftSku); Non-SaaS background (IT services/consulting, not SaaS)</t>
         </is>
       </c>
-      <c r="AN305" s="15" t="inlineStr"/>
+      <c r="AN305" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="15" t="inlineStr">
@@ -48628,10 +48624,8 @@
           <t>26.0</t>
         </is>
       </c>
-      <c r="AH306" s="15" t="inlineStr">
-        <is>
-          <t>53.4</t>
-        </is>
+      <c r="AH306" s="15" t="n">
+        <v>53.4</v>
       </c>
       <c r="AI306" s="15" t="inlineStr">
         <is>
@@ -48662,7 +48656,11 @@
           <t>No SaaS product experience; no high-volume sourcing metrics; short tenures; not a specialized recruiting coordinator</t>
         </is>
       </c>
-      <c r="AN306" s="15" t="inlineStr"/>
+      <c r="AN306" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="15" t="inlineStr">
@@ -48822,14 +48820,12 @@
           <t>20.0</t>
         </is>
       </c>
-      <c r="AH307" s="15" t="inlineStr">
-        <is>
-          <t>53.4</t>
-        </is>
+      <c r="AH307" s="15" t="n">
+        <v>53.4</v>
       </c>
       <c r="AI307" s="15" t="inlineStr">
         <is>
-          <t>37.45%</t>
+          <t>37.5%</t>
         </is>
       </c>
       <c r="AJ307" s="15" t="inlineStr">
@@ -48857,7 +48853,11 @@
           <t>Non-tech recruiting background, not SaaS/startup</t>
         </is>
       </c>
-      <c r="AN307" s="15" t="inlineStr"/>
+      <c r="AN307" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="15" t="inlineStr">
@@ -48964,7 +48964,7 @@
       </c>
       <c r="AI308" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ308" s="15" t="inlineStr">
@@ -48979,7 +48979,11 @@
       </c>
       <c r="AL308" s="15" t="inlineStr"/>
       <c r="AM308" s="15" t="inlineStr"/>
-      <c r="AN308" s="15" t="inlineStr"/>
+      <c r="AN308" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="15" t="inlineStr">
@@ -49101,30 +49105,20 @@
           <t>Profile not accessible</t>
         </is>
       </c>
-      <c r="AD309" s="15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AE309" s="15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AF309" s="15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AG309" s="15" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AH309" s="15" t="inlineStr">
-        <is>
-          <t>53.4</t>
-        </is>
+      <c r="AD309" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE309" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF309" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG309" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH309" s="15" t="n">
+        <v>53.4</v>
       </c>
       <c r="AI309" s="15" t="inlineStr">
         <is>
@@ -49138,7 +49132,7 @@
       </c>
       <c r="AK309" s="15" t="inlineStr">
         <is>
-          <t>Unable to Evaluate</t>
+          <t>Hard No</t>
         </is>
       </c>
       <c r="AL309" s="15" t="inlineStr"/>
@@ -49147,7 +49141,11 @@
           <t>LinkedIn Recruiter access denied</t>
         </is>
       </c>
-      <c r="AN309" s="15" t="inlineStr"/>
+      <c r="AN309" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -49290,34 +49288,24 @@
           <t>Auto-DQ</t>
         </is>
       </c>
-      <c r="AD310" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="AE310" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="AF310" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="AG310" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="AH310" t="inlineStr">
-        <is>
-          <t>53.4</t>
-        </is>
+      <c r="AD310" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE310" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF310" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG310" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH310" t="n">
+        <v>53.4</v>
       </c>
       <c r="AI310" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="AJ310" t="inlineStr">
@@ -49333,6 +49321,11 @@
       <c r="AM310" t="inlineStr">
         <is>
           <t>Career entirely in staffing agencies and IT services/non-product companies. No in-house recruiting coordinator experience at a product company. Adecco Group is a major staffing agency.</t>
+        </is>
+      </c>
+      <c r="AN310" t="inlineStr">
+        <is>
+          <t>TRUE</t>
         </is>
       </c>
     </row>
@@ -49497,14 +49490,12 @@
           <t>11.2</t>
         </is>
       </c>
-      <c r="AH311" t="inlineStr">
-        <is>
-          <t>53.4</t>
-        </is>
+      <c r="AH311" t="n">
+        <v>53.4</v>
       </c>
       <c r="AI311" t="inlineStr">
         <is>
-          <t>20.97%</t>
+          <t>21.0%</t>
         </is>
       </c>
       <c r="AJ311" t="inlineStr">
@@ -49530,6 +49521,11 @@
           <t>VOIS is telecom IT services; title mismatch (level too senior, wrong function)</t>
         </is>
       </c>
+      <c r="AN311" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" s="15" t="inlineStr">
@@ -49689,10 +49685,8 @@
           <t>19.9</t>
         </is>
       </c>
-      <c r="AH312" s="15" t="inlineStr">
-        <is>
-          <t>53.4</t>
-        </is>
+      <c r="AH312" s="15" t="n">
+        <v>53.4</v>
       </c>
       <c r="AI312" s="15" t="inlineStr">
         <is>
@@ -49725,7 +49719,11 @@
           <t>0% SaaS fit; non-tech traditional industry background (Adani); no Sales hiring exposure</t>
         </is>
       </c>
-      <c r="AN312" s="15" t="inlineStr"/>
+      <c r="AN312" s="15" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>